<commit_message>
feat: configure environment, rtk, mcp, and skills
</commit_message>
<xml_diff>
--- a/AI工具/Amazon Image Extractor/amazon_images_result.xlsx
+++ b/AI工具/Amazon Image Extractor/amazon_images_result.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K176"/>
+  <dimension ref="A1:K177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10432,6 +10432,63 @@
         </is>
       </c>
     </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>B0D4YSJJMG</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/81S7QZ-ca7L.jpg</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/41rjct8rfJL.jpg</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/71xEn4gsJjL.jpg</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/41TNkVZJDAL.jpg</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/81-yzpGyS4L.jpg</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/51UujBILidL.jpg</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/71.jpg</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/41OP1H5ikVL.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>